<commit_message>
Erick loans corrected per owner: R250 + R250 this week and next (not R500 + R500)
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
@@ -8907,10 +8907,10 @@
         <f>MAX(0,T8-U8)</f>
       </c>
       <c r="W8" s="4">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="X8" s="7">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="Y8" s="4">
         <f>MAX(0,1000-X8)</f>
@@ -12835,16 +12835,16 @@
         <v>2000</v>
       </c>
       <c r="G13" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H13" s="4">
-        <v>2000</v>
+        <v>1750</v>
       </c>
       <c r="I13" s="5">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="J13" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
@@ -12853,7 +12853,7 @@
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">paid</t>
+          <t xml:space="preserve">active</t>
         </is>
       </c>
     </row>
@@ -12887,16 +12887,16 @@
         <v>500</v>
       </c>
       <c r="G14" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H14" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="I14" s="5">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="J14" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
@@ -12905,7 +12905,7 @@
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">paid</t>
+          <t xml:space="preserve">active</t>
         </is>
       </c>
     </row>
@@ -13315,16 +13315,16 @@
         </is>
       </c>
       <c r="F25" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G25" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H25" s="4">
         <v>500</v>
       </c>
       <c r="I25" s="4">
-        <v>0</v>
+        <v>250</v>
       </c>
     </row>
     <row r="26">
@@ -13744,16 +13744,16 @@
         </is>
       </c>
       <c r="F36" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G36" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H36" s="4">
         <v>500</v>
       </c>
       <c r="I36" s="4">
-        <v>0</v>
+        <v>250</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
Auditor Excel: DEDUCTION NOTES column (why we deduct), dark gridlines, wider columns (v2026-09-30-5)
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
@@ -98,7 +98,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -121,36 +121,59 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1" vertical="top"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1" vertical="top"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -169,6 +192,15 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="center" horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8209,36 +8241,37 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="6" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
     <col min="8" max="8" width="6" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
     <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="11" max="11" width="11" customWidth="1"/>
     <col min="12" max="12" width="6" customWidth="1"/>
-    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
     <col min="14" max="14" width="6" customWidth="1"/>
-    <col min="15" max="15" width="10" customWidth="1"/>
+    <col min="15" max="15" width="11" customWidth="1"/>
     <col min="16" max="16" width="7" customWidth="1"/>
     <col min="17" max="17" width="11" customWidth="1"/>
-    <col min="18" max="18" width="11" customWidth="1"/>
-    <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="11" customWidth="1"/>
-    <col min="21" max="21" width="11" customWidth="1"/>
-    <col min="22" max="22" width="11" customWidth="1"/>
-    <col min="23" max="23" width="11" customWidth="1"/>
-    <col min="24" max="24" width="11" customWidth="1"/>
-    <col min="25" max="25" width="11" customWidth="1"/>
-    <col min="26" max="26" width="11" customWidth="1"/>
-    <col min="27" max="27" width="12" customWidth="1"/>
+    <col min="18" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="14" customWidth="1"/>
+    <col min="22" max="22" width="14" customWidth="1"/>
+    <col min="23" max="23" width="14" customWidth="1"/>
+    <col min="24" max="24" width="14" customWidth="1"/>
+    <col min="25" max="25" width="14" customWidth="1"/>
+    <col min="26" max="26" width="14" customWidth="1"/>
+    <col min="27" max="27" width="15" customWidth="1"/>
+    <col min="28" max="28" width="95" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Employee</t>
@@ -8342,8 +8375,13 @@
           <t xml:space="preserve">NET WAGE</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEDUCTION NOTES — why we are deducting (for the auditor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -8403,8 +8441,9 @@
       <c r="Y2" s="2"/>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
-    </row>
-    <row r="3">
+      <c r="AB2" s="2"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -8496,9 +8535,10 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Bhekizitha Maphosa</t>
         </is>
@@ -8581,9 +8621,10 @@
       <c r="AA4" s="13">
         <f>MAX(0,S4-Z4)</f>
       </c>
+      <c r="AB4" s="36"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Brian Ndlovu</t>
         </is>
@@ -8666,9 +8707,10 @@
       <c r="AA5" s="13">
         <f>MAX(0,S5-Z5)</f>
       </c>
+      <c r="AB5" s="36"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Daniel Motaung</t>
         </is>
@@ -8751,9 +8793,10 @@
       <c r="AA6" s="13">
         <f>MAX(0,S6-Z6)</f>
       </c>
+      <c r="AB6" s="36"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Erence Mngomezulu</t>
         </is>
@@ -8836,9 +8879,10 @@
       <c r="AA7" s="13">
         <f>MAX(0,S7-Z7)</f>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="AB7" s="36"/>
+    </row>
+    <row r="8" ht="97" customHeight="1">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Erick Mpho Molefe</t>
         </is>
@@ -8921,9 +8965,16 @@
       <c r="AA8" s="13">
         <f>MAX(0,S8-Z8)</f>
       </c>
+      <c r="AB8" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
+2. LOAN #1 R2 000,00 given 2026-08-08 (car repair): R250,00 deducted this week; R250,00 still owing → next payroll.
+3. LOAN #7 R500,00 given 2026-09-22 (cash advance requested by WhatsApp): R250,00 deducted this week; R250,00 still owing → next payroll.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Givemore Chifetete Kuziwa</t>
         </is>
@@ -9006,9 +9057,10 @@
       <c r="AA9" s="13">
         <f>MAX(0,S9-Z9)</f>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="AB9" s="36"/>
+    </row>
+    <row r="10" ht="151" customHeight="1">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
         </is>
@@ -9091,9 +9143,18 @@
       <c r="AA10" s="13">
         <f>MAX(0,S10-Z10)</f>
       </c>
+      <c r="AB10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. FIXED R260,00/week — Eggs, every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
+2. LOAN #2 R900,00 given 2026-08-11 (cash advance): R250,00 deducted this week; R100,00 still owing → next payroll.
+3. LOAN #3 R600,00 given 2026-08-16 (cash advance): R150,00 deducted this week (only what was left); now fully repaid — CLOSED, nothing further.
+4. LOAN #6 R600,00 given 2026-09-01 (children's school trip): R600,00 deducted this week; now fully repaid — CLOSED, nothing further.
+5. LOAN #8 R500,00 given 2026-09-22 (fuel / oil): R250,00 deducted this week; R250,00 still owing → next payroll.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">John Simbarashe Mhlanga</t>
         </is>
@@ -9176,9 +9237,10 @@
       <c r="AA11" s="13">
         <f>MAX(0,S11-Z11)</f>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="AB11" s="36"/>
+    </row>
+    <row r="12" ht="43" customHeight="1">
+      <c r="A12" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Joshua Motsamai Nteo</t>
         </is>
@@ -9261,9 +9323,14 @@
       <c r="AA12" s="13">
         <f>MAX(0,S12-Z12)</f>
       </c>
+      <c r="AB12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-09-26, ongoing until the owner ends it. Not a loan.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Lebo Lebo</t>
         </is>
@@ -9346,9 +9413,10 @@
       <c r="AA13" s="13">
         <f>MAX(0,S13-Z13)</f>
       </c>
+      <c r="AB13" s="36"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Patrick Ngozo</t>
         </is>
@@ -9431,9 +9499,10 @@
       <c r="AA14" s="13">
         <f>MAX(0,S14-Z14)</f>
       </c>
+      <c r="AB14" s="36"/>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Sharleen Ndlovu</t>
         </is>
@@ -9516,9 +9585,10 @@
       <c r="AA15" s="13">
         <f>MAX(0,S15-Z15)</f>
       </c>
+      <c r="AB15" s="36"/>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Solomon Moyo</t>
         </is>
@@ -9601,9 +9671,10 @@
       <c r="AA16" s="13">
         <f>MAX(0,S16-Z16)</f>
       </c>
+      <c r="AB16" s="36"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Takavaudza Chokuda</t>
         </is>
@@ -9686,9 +9757,10 @@
       <c r="AA17" s="13">
         <f>MAX(0,S17-Z17)</f>
       </c>
+      <c r="AB17" s="36"/>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Thandanani Nkala</t>
         </is>
@@ -9771,9 +9843,10 @@
       <c r="AA18" s="13">
         <f>MAX(0,S18-Z18)</f>
       </c>
+      <c r="AB18" s="36"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Thina Dyani</t>
         </is>
@@ -9856,9 +9929,10 @@
       <c r="AA19" s="13">
         <f>MAX(0,S19-Z19)</f>
       </c>
+      <c r="AB19" s="36"/>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Tsotlego Petrus Malakoane</t>
         </is>
@@ -9941,9 +10015,10 @@
       <c r="AA20" s="13">
         <f>MAX(0,S20-Z20)</f>
       </c>
+      <c r="AB20" s="36"/>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">GRAND TOTAL</t>
         </is>
@@ -10026,9 +10101,10 @@
       <c r="AA21" s="5">
         <f>SUM(AA4:AA20)</f>
       </c>
+      <c r="AB21" s="35"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -10056,6 +10132,7 @@
     <mergeCell ref="Y1:Y3"/>
     <mergeCell ref="Z1:Z3"/>
     <mergeCell ref="AA1:AA3"/>
+    <mergeCell ref="AB1:AB3"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -10063,19 +10140,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="13" customWidth="1"/>
-    <col min="12" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="95" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -10092,7 +10170,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Name</t>
@@ -10158,9 +10236,14 @@
           <t xml:space="preserve">NET WAGE</t>
         </is>
       </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEDUCTION NOTES — why we are deducting (for the auditor)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="0" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Bhekizitha Maphosa</t>
         </is>
@@ -10201,9 +10284,10 @@
       <c r="M5" s="13">
         <f>'Auditor Trail Linked'!AA4</f>
       </c>
+      <c r="N5" s="36"/>
     </row>
     <row r="6">
-      <c r="A6" s="0" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Brian Ndlovu</t>
         </is>
@@ -10244,9 +10328,10 @@
       <c r="M6" s="13">
         <f>'Auditor Trail Linked'!AA5</f>
       </c>
+      <c r="N6" s="36"/>
     </row>
     <row r="7">
-      <c r="A7" s="0" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Daniel Motaung</t>
         </is>
@@ -10287,9 +10372,10 @@
       <c r="M7" s="13">
         <f>'Auditor Trail Linked'!AA6</f>
       </c>
+      <c r="N7" s="36"/>
     </row>
     <row r="8">
-      <c r="A8" s="0" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Erence Mngomezulu</t>
         </is>
@@ -10330,9 +10416,10 @@
       <c r="M8" s="13">
         <f>'Auditor Trail Linked'!AA7</f>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="0" t="inlineStr">
+      <c r="N8" s="36"/>
+    </row>
+    <row r="9" ht="97" customHeight="1">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Erick Mpho Molefe</t>
         </is>
@@ -10373,9 +10460,16 @@
       <c r="M9" s="13">
         <f>'Auditor Trail Linked'!AA8</f>
       </c>
+      <c r="N9" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
+2. LOAN #1 R2 000,00 given 2026-08-08 (car repair): R250,00 deducted this week; R250,00 still owing → next payroll.
+3. LOAN #7 R500,00 given 2026-09-22 (cash advance requested by WhatsApp): R250,00 deducted this week; R250,00 still owing → next payroll.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="0" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Givemore Chifetete Kuziwa</t>
         </is>
@@ -10416,9 +10510,10 @@
       <c r="M10" s="13">
         <f>'Auditor Trail Linked'!AA9</f>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="N10" s="36"/>
+    </row>
+    <row r="11" ht="151" customHeight="1">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
         </is>
@@ -10459,9 +10554,18 @@
       <c r="M11" s="13">
         <f>'Auditor Trail Linked'!AA10</f>
       </c>
+      <c r="N11" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. FIXED R260,00/week — Eggs, every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
+2. LOAN #2 R900,00 given 2026-08-11 (cash advance): R250,00 deducted this week; R100,00 still owing → next payroll.
+3. LOAN #3 R600,00 given 2026-08-16 (cash advance): R150,00 deducted this week (only what was left); now fully repaid — CLOSED, nothing further.
+4. LOAN #6 R600,00 given 2026-09-01 (children's school trip): R600,00 deducted this week; now fully repaid — CLOSED, nothing further.
+5. LOAN #8 R500,00 given 2026-09-22 (fuel / oil): R250,00 deducted this week; R250,00 still owing → next payroll.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="0" t="inlineStr">
+      <c r="A12" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">John Simbarashe Mhlanga</t>
         </is>
@@ -10502,9 +10606,10 @@
       <c r="M12" s="13">
         <f>'Auditor Trail Linked'!AA11</f>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="0" t="inlineStr">
+      <c r="N12" s="36"/>
+    </row>
+    <row r="13" ht="43" customHeight="1">
+      <c r="A13" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Joshua Motsamai Nteo</t>
         </is>
@@ -10545,9 +10650,14 @@
       <c r="M13" s="13">
         <f>'Auditor Trail Linked'!AA12</f>
       </c>
+      <c r="N13" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-09-26, ongoing until the owner ends it. Not a loan.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="0" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Lebo Lebo</t>
         </is>
@@ -10588,9 +10698,10 @@
       <c r="M14" s="13">
         <f>'Auditor Trail Linked'!AA13</f>
       </c>
+      <c r="N14" s="36"/>
     </row>
     <row r="15">
-      <c r="A15" s="0" t="inlineStr">
+      <c r="A15" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Patrick Ngozo</t>
         </is>
@@ -10631,9 +10742,10 @@
       <c r="M15" s="13">
         <f>'Auditor Trail Linked'!AA14</f>
       </c>
+      <c r="N15" s="36"/>
     </row>
     <row r="16">
-      <c r="A16" s="0" t="inlineStr">
+      <c r="A16" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Sharleen Ndlovu</t>
         </is>
@@ -10674,9 +10786,10 @@
       <c r="M16" s="13">
         <f>'Auditor Trail Linked'!AA15</f>
       </c>
+      <c r="N16" s="36"/>
     </row>
     <row r="17">
-      <c r="A17" s="0" t="inlineStr">
+      <c r="A17" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Solomon Moyo</t>
         </is>
@@ -10717,9 +10830,10 @@
       <c r="M17" s="13">
         <f>'Auditor Trail Linked'!AA16</f>
       </c>
+      <c r="N17" s="36"/>
     </row>
     <row r="18">
-      <c r="A18" s="0" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Takavaudza Chokuda</t>
         </is>
@@ -10760,9 +10874,10 @@
       <c r="M18" s="13">
         <f>'Auditor Trail Linked'!AA17</f>
       </c>
+      <c r="N18" s="36"/>
     </row>
     <row r="19">
-      <c r="A19" s="0" t="inlineStr">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Thandanani Nkala</t>
         </is>
@@ -10803,9 +10918,10 @@
       <c r="M19" s="13">
         <f>'Auditor Trail Linked'!AA18</f>
       </c>
+      <c r="N19" s="36"/>
     </row>
     <row r="20">
-      <c r="A20" s="0" t="inlineStr">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Thina Dyani</t>
         </is>
@@ -10846,9 +10962,10 @@
       <c r="M20" s="13">
         <f>'Auditor Trail Linked'!AA19</f>
       </c>
+      <c r="N20" s="36"/>
     </row>
     <row r="21">
-      <c r="A21" s="0" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Tsotlego Petrus Malakoane</t>
         </is>
@@ -10889,9 +11006,10 @@
       <c r="M21" s="13">
         <f>'Auditor Trail Linked'!AA20</f>
       </c>
+      <c r="N21" s="36"/>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">GRAND TOTAL</t>
         </is>
@@ -10932,11 +11050,12 @@
       <c r="M22" s="5">
         <f>SUM(M5:M21)</f>
       </c>
+      <c r="N22" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Auditor note: only actual deductions this week; Isaac next week #6 R360 + #8 R500 in full (v2026-10-01-2)
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
@@ -5235,16 +5235,6 @@
         </is>
       </c>
       <c r="U67" s="6"/>
-      <c r="W67" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#10315 Manual overlap review: the same employee has another overlapping entry on 2026-09-30 for 07:00-16:00.</t>
-        </is>
-      </c>
-      <c r="X67" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#10315 STILL OPEN — no decision recorded yet (claimed hours used)</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" s="0">
@@ -9054,8 +9044,8 @@
       <c r="AB8" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">1. FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
-2. LOAN #1 R2 000,00 given 2026-08-08 (car repair): R250,00 deducted this week; R250,00 still owing → R250,00/week from next payroll.
-3. LOAN #7 R500,00 given 2026-09-22 (cash advance requested by WhatsApp): R250,00 deducted this week; R250,00 still owing → R250,00/week from next payroll.</t>
+2. LOAN #1 R2 000,00 given 2026-08-08 (car repair): R250,00 deducted this week; R250,00 still owing — carried to the next payroll.
+3. LOAN #7 R500,00 given 2026-09-22 (cash advance requested by WhatsApp): R250,00 deducted this week; R250,00 still owing — carried to the next payroll.</t>
         </is>
       </c>
     </row>
@@ -9145,7 +9135,7 @@
       </c>
       <c r="AB9" s="36"/>
     </row>
-    <row r="10" ht="151" customHeight="1">
+    <row r="10" ht="124" customHeight="1">
       <c r="A10" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
@@ -9234,8 +9224,7 @@
           <t xml:space="preserve">1. FIXED R260,00/week — Eggs, every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
 2. LOAN #2 R900,00 given 2026-08-11 (cash advance): R350,00 deducted this week; now fully repaid — CLOSED, nothing further.
 3. LOAN #3 R600,00 given 2026-08-16 (cash advance): R150,00 deducted this week (only what was left); now fully repaid — CLOSED, nothing further.
-4. LOAN #6 R600,00 given 2026-09-01 (children's school trip): R240,00 deducted this week; R360,00 still owing → R250,00/week from next payroll.
-5. LOAN #8 R500,00 given 2026-09-22 (fuel / oil): NOTHING taken this week by owner decision — R500,00 still owing, R250,00/week from the next payroll.</t>
+4. LOAN #6 R600,00 given 2026-09-01 (children's school trip): R240,00 deducted this week; R360,00 still owing — carried to the next payroll.</t>
         </is>
       </c>
     </row>
@@ -10549,8 +10538,8 @@
       <c r="N9" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">1. FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
-2. LOAN #1 R2 000,00 given 2026-08-08 (car repair): R250,00 deducted this week; R250,00 still owing → R250,00/week from next payroll.
-3. LOAN #7 R500,00 given 2026-09-22 (cash advance requested by WhatsApp): R250,00 deducted this week; R250,00 still owing → R250,00/week from next payroll.</t>
+2. LOAN #1 R2 000,00 given 2026-08-08 (car repair): R250,00 deducted this week; R250,00 still owing — carried to the next payroll.
+3. LOAN #7 R500,00 given 2026-09-22 (cash advance requested by WhatsApp): R250,00 deducted this week; R250,00 still owing — carried to the next payroll.</t>
         </is>
       </c>
     </row>
@@ -10598,7 +10587,7 @@
       </c>
       <c r="N10" s="36"/>
     </row>
-    <row r="11" ht="151" customHeight="1">
+    <row r="11" ht="124" customHeight="1">
       <c r="A11" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
@@ -10645,8 +10634,7 @@
           <t xml:space="preserve">1. FIXED R260,00/week — Eggs, every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
 2. LOAN #2 R900,00 given 2026-08-11 (cash advance): R350,00 deducted this week; now fully repaid — CLOSED, nothing further.
 3. LOAN #3 R600,00 given 2026-08-16 (cash advance): R150,00 deducted this week (only what was left); now fully repaid — CLOSED, nothing further.
-4. LOAN #6 R600,00 given 2026-09-01 (children's school trip): R240,00 deducted this week; R360,00 still owing → R250,00/week from next payroll.
-5. LOAN #8 R500,00 given 2026-09-22 (fuel / oil): NOTHING taken this week by owner decision — R500,00 still owing, R250,00/week from the next payroll.</t>
+4. LOAN #6 R600,00 given 2026-09-01 (children's school trip): R240,00 deducted this week; R360,00 still owing — carried to the next payroll.</t>
         </is>
       </c>
     </row>
@@ -11792,27 +11780,27 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN</t>
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
       <c r="B14" s="17">
-        <v>10315</v>
+        <v>10168</v>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lebo Lebo</t>
+          <t xml:space="preserve">Patrick Ngozo</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-30</t>
+          <t xml:space="preserve">2026-09-25</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Sunbet</t>
+          <t xml:space="preserve">05:00–07:00 Pretoria Country Club</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr">
@@ -11822,202 +11810,218 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-30 for 07:00-16:00.</t>
+          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-25 for 05:00-07:00.</t>
         </is>
       </c>
       <c r="H14" s="17"/>
       <c r="I14" s="18">
-        <v>9</v>
-      </c>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
+        <v>2</v>
+      </c>
+      <c r="J14" s="18">
+        <v>2</v>
+      </c>
+      <c r="K14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve adjusted</t>
+        </is>
+      </c>
+      <c r="L14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-27 14:15:39</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B15" s="20">
-        <v>10168</v>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="B15" s="17">
+        <v>10173</v>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Patrick Ngozo</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-25</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">05:00–07:00 Pretoria Country Club</t>
         </is>
       </c>
-      <c r="F15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manual overlap review</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-25 for 05:00-07:00.</t>
-        </is>
-      </c>
-      <c r="H15" s="20"/>
-      <c r="I15" s="21">
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALREADY PAID — this claim is covered by what was paid</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patrick was paid Fri 25 Sep 2026 06:30–16:00 · Pretoria Country Club (Pretoria) · Normal · "Set up Golf ⛳️  course" · 9.50 h × R95,00 = R902,50 (payroll 2026-09-19). He now claims 05:00–07:00 · Pretoria Country Club (Pretoria) · Normal · "Set up golf day" · 2.00 h for the same day. Same work type, but the rate paid (R95,00/h) differs from the rule (R95,00/h). • Rate correction on the paid hours 06:30–07:00: 0.50 h — worth R47,50 at the correct rule, R902,50 was paid → −R855,00 • Extra hours 05:00–06:30: 1.50 h → R142,50 What was paid (R902,50) already covers this claim (R190,00 at the correct rule). Nothing more is due: R0,00. Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
+        </is>
+      </c>
+      <c r="H15" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="I15" s="18">
         <v>2</v>
       </c>
-      <c r="J15" s="21">
-        <v>2</v>
-      </c>
-      <c r="K15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L15" s="20" t="inlineStr">
+      <c r="J15" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve additional hours only</t>
+        </is>
+      </c>
+      <c r="L15" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-27 14:15:39</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Approved.</t>
+      <c r="M15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-27 14:20:06</t>
+        </is>
+      </c>
+      <c r="N15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner 27 Sep: already paid 06:30–16:00 on #9839 (R902,50). Only the uncovered 05:00–06:30 = 1,5 h × R95 = R142,50 is due on #9870 — row set to R142,50.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B16" s="20">
-        <v>10173</v>
-      </c>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="B16" s="17">
+        <v>10189</v>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Patrick Ngozo</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-25</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">05:00–07:00 Pretoria Country Club</t>
-        </is>
-      </c>
-      <c r="F16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALREADY PAID — this claim is covered by what was paid</t>
-        </is>
-      </c>
-      <c r="G16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Patrick was paid Fri 25 Sep 2026 06:30–16:00 · Pretoria Country Club (Pretoria) · Normal · "Set up Golf ⛳️  course" · 9.50 h × R95,00 = R902,50 (payroll 2026-09-19). He now claims 05:00–07:00 · Pretoria Country Club (Pretoria) · Normal · "Set up golf day" · 2.00 h for the same day. Same work type, but the rate paid (R95,00/h) differs from the rule (R95,00/h). • Rate correction on the paid hours 06:30–07:00: 0.50 h — worth R47,50 at the correct rule, R902,50 was paid → −R855,00 • Extra hours 05:00–06:30: 1.50 h → R142,50 What was paid (R902,50) already covers this claim (R190,00 at the correct rule). Nothing more is due: R0,00. Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
-        </is>
-      </c>
-      <c r="H16" s="21">
-        <v>1.5</v>
-      </c>
-      <c r="I16" s="21">
-        <v>2</v>
-      </c>
-      <c r="J16" s="21">
-        <v>1.5</v>
-      </c>
-      <c r="K16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve additional hours only</t>
-        </is>
-      </c>
-      <c r="L16" s="20" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06:30–16:00 Wearhouse</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+        </is>
+      </c>
+      <c r="H16" s="17"/>
+      <c r="I16" s="18">
+        <v>9.5</v>
+      </c>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L16" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-27 14:20:06</t>
-        </is>
-      </c>
-      <c r="N16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Owner 27 Sep: already paid 06:30–16:00 on #9839 (R902,50). Only the uncovered 05:00–06:30 = 1,5 h × R95 = R142,50 is due on #9870 — row set to R142,50.</t>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29 12:53:11</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9878 R795,00 → R731,25 (Warehouse: 9.5 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 9 h × R81,25)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B17" s="20">
-        <v>10189</v>
-      </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="B17" s="17">
+        <v>10234</v>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Patrick Ngozo</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06:30–16:00 Wearhouse</t>
-        </is>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06:30–16:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
-      <c r="G17" s="20" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
         </is>
       </c>
-      <c r="H17" s="20"/>
-      <c r="I17" s="21">
+      <c r="H17" s="17"/>
+      <c r="I17" s="18">
         <v>9.5</v>
       </c>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20" t="inlineStr">
+      <c r="J17" s="17"/>
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
         </is>
       </c>
-      <c r="L17" s="20" t="inlineStr">
+      <c r="L17" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M17" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29 12:53:11</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9878 R795,00 → R731,25 (Warehouse: 9.5 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 9 h × R81,25)</t>
+      <c r="M17" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-30 02:54:31</t>
+        </is>
+      </c>
+      <c r="N17" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Event/Venue rate chosen — shift #9902 R795,00 → R902,50 (Venue/event: 9.5 h × R95)</t>
         </is>
       </c>
     </row>
@@ -12028,21 +12032,21 @@
         </is>
       </c>
       <c r="B18" s="20">
-        <v>10234</v>
+        <v>10253</v>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Ngozo</t>
+          <t xml:space="preserve">Solomon Moyo</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-09-29</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">06:30–16:00 Warehouse</t>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
@@ -12057,27 +12061,27 @@
       </c>
       <c r="H18" s="20"/>
       <c r="I18" s="21">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="J18" s="20"/>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve original</t>
+          <t xml:space="preserve">approve adjusted</t>
         </is>
       </c>
       <c r="L18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bernie Burness</t>
+          <t xml:space="preserve">Bernie Burness (via assistant)</t>
         </is>
       </c>
       <c r="M18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-30 02:54:31</t>
+          <t xml:space="preserve">2026-09-30 07:34:12</t>
         </is>
       </c>
       <c r="N18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Event/Venue rate chosen — shift #9902 R795,00 → R902,50 (Venue/event: 9.5 h × R95)</t>
+          <t xml:space="preserve">Owner 30 Sep 2026: rate set by team/date rule (Sunbet set-up = event; same team same day = same rate). See row note.</t>
         </is>
       </c>
     </row>
@@ -12088,486 +12092,488 @@
         </is>
       </c>
       <c r="B19" s="23">
-        <v>10253</v>
+        <v>10180</v>
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solomon Moyo</t>
+          <t xml:space="preserve">Takavaudza Chokuda</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-29</t>
+          <t xml:space="preserve">2026-09-26</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">06:00–13:00 Warehouse</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+          <t xml:space="preserve">Crew pattern — 4 of 5 at a venue, this one says Warehouse</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+          <t xml:space="preserve">CREW PATTERN: 4 of 5 workers were at a venue on Sat 26 Sep 2026 (Brooklyn, Brooklyn pretoria, Sonop, SONOP) — Takavaudza Chokuda says Warehouse for 7.00 h. Check he was not at the venue (R95/h would be due).</t>
         </is>
       </c>
       <c r="H19" s="23"/>
       <c r="I19" s="24">
+        <v>7</v>
+      </c>
+      <c r="J19" s="24">
+        <v>7</v>
+      </c>
+      <c r="K19" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M19" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28 16:09:08</t>
+        </is>
+      </c>
+      <c r="N19" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE — R81,25/h chosen by Bernie Burness for draft #930 — will pay R568,75 when final-submitted (Warehouse: 7 h × R81,25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B20" s="23">
+        <v>10276</v>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takavaudza Chokuda</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-27</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–12:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crew pattern — 3 of 4 at a venue, this one says Warehouse</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CREW PATTERN: 3 of 4 workers were at a venue on Sun 27 Sep 2026 (Sandton Convention Centre and The Capital, Conversation center Sandton/ Capital hotel, Sandton convention centre) — Takavaudza Chokuda says Warehouse for 5.00 h. Check he was not at the venue (R95/h would be due).</t>
+        </is>
+      </c>
+      <c r="H20" s="23"/>
+      <c r="I20" s="24">
+        <v>5</v>
+      </c>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness (via assistant)</t>
+        </is>
+      </c>
+      <c r="M20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-30 07:34:48</t>
+        </is>
+      </c>
+      <c r="N20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner 27/28 Sep: Taka Sunday warehouse 07:00–12:00 at venue Sunday rate (R114) then house 12:30 — already ruled and priced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B21" s="23">
+        <v>10190</v>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takavaudza Chokuda</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Wanderas, Orlando pirates</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse claimed — but the entry names “Johannesburg”</t>
+        </is>
+      </c>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “Johannesburg”: Takavaudza Chokuda selected Warehouse Team at “Wanderas, Orlando pirates” for 9.00 h on Mon 28 Sep 2026, but wrote “Johannesburg” — that is a venue, not the warehouse. 5 workers were at a venue that day (Protea hotel wanderer, ORLANDO &amp; WANDERERS, Sonop Pretoria and Wanderers, Sonop Pretoria/ Protea hotel, Orlando stadium). If he was at “Johannesburg”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+        </is>
+      </c>
+      <c r="H21" s="23"/>
+      <c r="I21" s="24">
         <v>9</v>
       </c>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L19" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness (via assistant)</t>
-        </is>
-      </c>
-      <c r="M19" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-30 07:34:12</t>
-        </is>
-      </c>
-      <c r="N19" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Owner 30 Sep 2026: rate set by team/date rule (Sunbet set-up = event; same team same day = same rate). See row note.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="26" t="inlineStr">
+      <c r="J21" s="24">
+        <v>9</v>
+      </c>
+      <c r="K21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29 12:54:03</t>
+        </is>
+      </c>
+      <c r="N21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VENUE — R95/h chosen by Bernie Burness for draft #957 — will pay R855,00 when final-submitted (Venue/event: 9 h × R95) — worker selected "Warehouse Team"; office overrides to Venue</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B20" s="26">
-        <v>10180</v>
-      </c>
-      <c r="C20" s="26" t="inlineStr">
+      <c r="B22" s="23">
+        <v>10151</v>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">Takavaudza Chokuda</t>
         </is>
       </c>
-      <c r="D20" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-26</t>
-        </is>
-      </c>
-      <c r="E20" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06:00–13:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F20" s="26" t="inlineStr">
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18:00–21:00 FNB stadium</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse claimed — but the entry names “Johannesburg”</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “Johannesburg”: Takavaudza Chokuda selected Warehouse Team at “FNB stadium” for 6.00 h on Tue 29 Sep 2026, but wrote “Johannesburg” — that is a venue, not the warehouse. If he was at “Johannesburg”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+        </is>
+      </c>
+      <c r="H22" s="23"/>
+      <c r="I22" s="24">
+        <v>3</v>
+      </c>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28 16:08:29</t>
+        </is>
+      </c>
+      <c r="N22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Event/Venue rate chosen — shift #399 R540,00 → R570,00 (Venue/event: 6 h × R95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B23" s="23">
+        <v>10225</v>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takavaudza Chokuda</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse claimed — but the entry names “gardens”</t>
+        </is>
+      </c>
+      <c r="G23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “gardens”: Takavaudza Chokuda selected Warehouse Team at “Warehouse” for 9.00 h on Tue 29 Sep 2026, but wrote “gardens” — that is a venue, not the warehouse. If he was at “gardens”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+        </is>
+      </c>
+      <c r="H23" s="23"/>
+      <c r="I23" s="24">
+        <v>9</v>
+      </c>
+      <c r="J23" s="24">
+        <v>9</v>
+      </c>
+      <c r="K23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29 16:34:25</t>
+        </is>
+      </c>
+      <c r="N23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE — R81,25/h chosen by Bernie Burness for draft #981 — will pay R690,63 when final-submitted (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B24" s="23">
+        <v>10226</v>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takavaudza Chokuda</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-30</t>
+        </is>
+      </c>
+      <c r="E24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Sunbet</t>
+        </is>
+      </c>
+      <c r="F24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse claimed — but the entry names “Pretoria”</t>
+        </is>
+      </c>
+      <c r="G24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “Pretoria”: Takavaudza Chokuda selected Warehouse Team at “Sunbet” for 9.00 h on Wed 30 Sep 2026, but wrote “Pretoria” — that is a venue, not the warehouse. Other workers were at SunBet Arena Pretoria that day. If he was at “Pretoria”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+        </is>
+      </c>
+      <c r="H24" s="23"/>
+      <c r="I24" s="24">
+        <v>9</v>
+      </c>
+      <c r="J24" s="24">
+        <v>9</v>
+      </c>
+      <c r="K24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29 16:34:28</t>
+        </is>
+      </c>
+      <c r="N24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VENUE — R95/h chosen by Bernie Burness for draft #982 — will pay R855,00 when final-submitted (Venue/event: 9 h × R95) — worker selected "Warehouse Team"; office overrides to Venue</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B25" s="23">
+        <v>10227</v>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takavaudza Chokuda</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="E25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">Crew pattern — 4 of 5 at a venue, this one says Warehouse</t>
         </is>
       </c>
-      <c r="G20" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CREW PATTERN: 4 of 5 workers were at a venue on Sat 26 Sep 2026 (Brooklyn, Brooklyn pretoria, Sonop, SONOP) — Takavaudza Chokuda says Warehouse for 7.00 h. Check he was not at the venue (R95/h would be due).</t>
-        </is>
-      </c>
-      <c r="H20" s="26"/>
-      <c r="I20" s="27">
-        <v>7</v>
-      </c>
-      <c r="J20" s="27">
-        <v>7</v>
-      </c>
-      <c r="K20" s="26" t="inlineStr">
+      <c r="G25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CREW PATTERN: 4 of 5 workers were at a venue on Thu 1 Oct 2026 (Homecoming, Botanical Gardens, Pretoria Botanical Gardens) — Takavaudza Chokuda says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
+        </is>
+      </c>
+      <c r="H25" s="23"/>
+      <c r="I25" s="24">
+        <v>9</v>
+      </c>
+      <c r="J25" s="24">
+        <v>9</v>
+      </c>
+      <c r="K25" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
         </is>
       </c>
-      <c r="L20" s="26" t="inlineStr">
+      <c r="L25" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M20" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-28 16:09:08</t>
-        </is>
-      </c>
-      <c r="N20" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WAREHOUSE — R81,25/h chosen by Bernie Burness for draft #930 — will pay R568,75 when final-submitted (Warehouse: 7 h × R81,25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="M25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29 16:35:11</t>
+        </is>
+      </c>
+      <c r="N25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VENUE — R95/h chosen by Bernie Burness for draft #983 — will pay R855,00 when final-submitted (Venue/event: 9 h × R95) — worker selected "Warehouse Team"; office overrides to Venue</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B21" s="26">
-        <v>10276</v>
-      </c>
-      <c r="C21" s="26" t="inlineStr">
+      <c r="B26" s="23">
+        <v>10228</v>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">Takavaudza Chokuda</t>
         </is>
       </c>
-      <c r="D21" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-27</t>
-        </is>
-      </c>
-      <c r="E21" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–12:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F21" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Crew pattern — 3 of 4 at a venue, this one says Warehouse</t>
-        </is>
-      </c>
-      <c r="G21" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CREW PATTERN: 3 of 4 workers were at a venue on Sun 27 Sep 2026 (Sandton Convention Centre and The Capital, Conversation center Sandton/ Capital hotel, Sandton convention centre) — Takavaudza Chokuda says Warehouse for 5.00 h. Check he was not at the venue (R95/h would be due).</t>
-        </is>
-      </c>
-      <c r="H21" s="26"/>
-      <c r="I21" s="27">
-        <v>5</v>
-      </c>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26" t="inlineStr">
+      <c r="D26" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-02</t>
+        </is>
+      </c>
+      <c r="E26" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F26" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crew pattern — 4 of 5 at a venue, this one says Warehouse</t>
+        </is>
+      </c>
+      <c r="G26" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CREW PATTERN: 4 of 5 workers were at a venue on Fri 2 Oct 2026 (Cielo, Benoni, Pretoria Botanical Gardens, ONE WOMAN SHOW) — Takavaudza Chokuda says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
+        </is>
+      </c>
+      <c r="H26" s="23"/>
+      <c r="I26" s="24">
+        <v>9</v>
+      </c>
+      <c r="J26" s="24">
+        <v>9</v>
+      </c>
+      <c r="K26" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
         </is>
       </c>
-      <c r="L21" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness (via assistant)</t>
-        </is>
-      </c>
-      <c r="M21" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-30 07:34:48</t>
-        </is>
-      </c>
-      <c r="N21" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Owner 27/28 Sep: Taka Sunday warehouse 07:00–12:00 at venue Sunday rate (R114) then house 12:30 — already ruled and priced.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B22" s="26">
-        <v>10190</v>
-      </c>
-      <c r="C22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Takavaudza Chokuda</t>
-        </is>
-      </c>
-      <c r="D22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-28</t>
-        </is>
-      </c>
-      <c r="E22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Wanderas, Orlando pirates</t>
-        </is>
-      </c>
-      <c r="F22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse claimed — but the entry names “Johannesburg”</t>
-        </is>
-      </c>
-      <c r="G22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “Johannesburg”: Takavaudza Chokuda selected Warehouse Team at “Wanderas, Orlando pirates” for 9.00 h on Mon 28 Sep 2026, but wrote “Johannesburg” — that is a venue, not the warehouse. 5 workers were at a venue that day (Protea hotel wanderer, ORLANDO &amp; WANDERERS, Sonop Pretoria and Wanderers, Sonop Pretoria/ Protea hotel, Orlando stadium). If he was at “Johannesburg”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
-        </is>
-      </c>
-      <c r="H22" s="26"/>
-      <c r="I22" s="27">
-        <v>9</v>
-      </c>
-      <c r="J22" s="27">
-        <v>9</v>
-      </c>
-      <c r="K22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L22" s="26" t="inlineStr">
+      <c r="L26" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29 12:54:03</t>
-        </is>
-      </c>
-      <c r="N22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VENUE — R95/h chosen by Bernie Burness for draft #957 — will pay R855,00 when final-submitted (Venue/event: 9 h × R95) — worker selected "Warehouse Team"; office overrides to Venue</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B23" s="26">
-        <v>10151</v>
-      </c>
-      <c r="C23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Takavaudza Chokuda</t>
-        </is>
-      </c>
-      <c r="D23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29</t>
-        </is>
-      </c>
-      <c r="E23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18:00–21:00 FNB stadium</t>
-        </is>
-      </c>
-      <c r="F23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse claimed — but the entry names “Johannesburg”</t>
-        </is>
-      </c>
-      <c r="G23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “Johannesburg”: Takavaudza Chokuda selected Warehouse Team at “FNB stadium” for 6.00 h on Tue 29 Sep 2026, but wrote “Johannesburg” — that is a venue, not the warehouse. If he was at “Johannesburg”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
-        </is>
-      </c>
-      <c r="H23" s="26"/>
-      <c r="I23" s="27">
-        <v>3</v>
-      </c>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-28 16:08:29</t>
-        </is>
-      </c>
-      <c r="N23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Event/Venue rate chosen — shift #399 R540,00 → R570,00 (Venue/event: 6 h × R95)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B24" s="26">
-        <v>10225</v>
-      </c>
-      <c r="C24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Takavaudza Chokuda</t>
-        </is>
-      </c>
-      <c r="D24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29</t>
-        </is>
-      </c>
-      <c r="E24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse claimed — but the entry names “gardens”</t>
-        </is>
-      </c>
-      <c r="G24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “gardens”: Takavaudza Chokuda selected Warehouse Team at “Warehouse” for 9.00 h on Tue 29 Sep 2026, but wrote “gardens” — that is a venue, not the warehouse. If he was at “gardens”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
-        </is>
-      </c>
-      <c r="H24" s="26"/>
-      <c r="I24" s="27">
-        <v>9</v>
-      </c>
-      <c r="J24" s="27">
-        <v>9</v>
-      </c>
-      <c r="K24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29 16:34:25</t>
-        </is>
-      </c>
-      <c r="N24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WAREHOUSE — R81,25/h chosen by Bernie Burness for draft #981 — will pay R690,63 when final-submitted (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B25" s="26">
-        <v>10226</v>
-      </c>
-      <c r="C25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Takavaudza Chokuda</t>
-        </is>
-      </c>
-      <c r="D25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-30</t>
-        </is>
-      </c>
-      <c r="E25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Sunbet</t>
-        </is>
-      </c>
-      <c r="F25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse claimed — but the entry names “Pretoria”</t>
-        </is>
-      </c>
-      <c r="G25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “Pretoria”: Takavaudza Chokuda selected Warehouse Team at “Sunbet” for 9.00 h on Wed 30 Sep 2026, but wrote “Pretoria” — that is a venue, not the warehouse. Other workers were at SunBet Arena Pretoria that day. If he was at “Pretoria”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
-        </is>
-      </c>
-      <c r="H25" s="26"/>
-      <c r="I25" s="27">
-        <v>9</v>
-      </c>
-      <c r="J25" s="27">
-        <v>9</v>
-      </c>
-      <c r="K25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29 16:34:28</t>
-        </is>
-      </c>
-      <c r="N25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VENUE — R95/h chosen by Bernie Burness for draft #982 — will pay R855,00 when final-submitted (Venue/event: 9 h × R95) — worker selected "Warehouse Team"; office overrides to Venue</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B26" s="26">
-        <v>10227</v>
-      </c>
-      <c r="C26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Takavaudza Chokuda</t>
-        </is>
-      </c>
-      <c r="D26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-01</t>
-        </is>
-      </c>
-      <c r="E26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Crew pattern — 4 of 5 at a venue, this one says Warehouse</t>
-        </is>
-      </c>
-      <c r="G26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CREW PATTERN: 4 of 5 workers were at a venue on Thu 1 Oct 2026 (Homecoming, Botanical Gardens, Pretoria Botanical Gardens) — Takavaudza Chokuda says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
-        </is>
-      </c>
-      <c r="H26" s="26"/>
-      <c r="I26" s="27">
-        <v>9</v>
-      </c>
-      <c r="J26" s="27">
-        <v>9</v>
-      </c>
-      <c r="K26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29 16:35:11</t>
-        </is>
-      </c>
-      <c r="N26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VENUE — R95/h chosen by Bernie Burness for draft #983 — will pay R855,00 when final-submitted (Venue/event: 9 h × R95) — worker selected "Warehouse Team"; office overrides to Venue</t>
+      <c r="M26" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29 16:35:22</t>
+        </is>
+      </c>
+      <c r="N26" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VENUE — R95/h chosen by Bernie Burness for draft #984 — will pay R855,00 when final-submitted (Venue/event: 9 h × R95) — worker selected "Warehouse Team"; office overrides to Venue</t>
         </is>
       </c>
     </row>
@@ -12578,176 +12584,114 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <v>10228</v>
+        <v>10301</v>
       </c>
       <c r="C27" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Takavaudza Chokuda</t>
+          <t xml:space="preserve">Thandanani Nkala</t>
         </is>
       </c>
       <c r="D27" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-02</t>
+          <t xml:space="preserve">2026-09-28</t>
         </is>
       </c>
       <c r="E27" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">07:00–16:00 Orlando Amstel Arena/Wanderers Stadium/Warehouse</t>
         </is>
       </c>
       <c r="F27" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crew pattern — 4 of 5 at a venue, this one says Warehouse</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G27" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">CREW PATTERN: 4 of 5 workers were at a venue on Fri 2 Oct 2026 (Cielo, Benoni, Pretoria Botanical Gardens, ONE WOMAN SHOW) — Takavaudza Chokuda says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
         </is>
       </c>
       <c r="H27" s="26"/>
       <c r="I27" s="27">
         <v>9</v>
       </c>
-      <c r="J27" s="27">
+      <c r="J27" s="26"/>
+      <c r="K27" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve adjusted</t>
+        </is>
+      </c>
+      <c r="L27" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness (via assistant)</t>
+        </is>
+      </c>
+      <c r="M27" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-30 07:34:12</t>
+        </is>
+      </c>
+      <c r="N27" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner 30 Sep 2026: rate set by team/date rule (Sunbet set-up = event; same team same day = same rate). See row note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B28" s="26">
+        <v>10299</v>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thandanani Nkala</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+        </is>
+      </c>
+      <c r="G28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+        </is>
+      </c>
+      <c r="H28" s="26"/>
+      <c r="I28" s="27">
         <v>9</v>
       </c>
-      <c r="K27" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L27" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M27" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29 16:35:22</t>
-        </is>
-      </c>
-      <c r="N27" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VENUE — R95/h chosen by Bernie Burness for draft #984 — will pay R855,00 when final-submitted (Venue/event: 9 h × R95) — worker selected "Warehouse Team"; office overrides to Venue</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B28" s="29">
-        <v>10301</v>
-      </c>
-      <c r="C28" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thandanani Nkala</t>
-        </is>
-      </c>
-      <c r="D28" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-28</t>
-        </is>
-      </c>
-      <c r="E28" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Orlando Amstel Arena/Wanderers Stadium/Warehouse</t>
-        </is>
-      </c>
-      <c r="F28" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
-        </is>
-      </c>
-      <c r="G28" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
-        </is>
-      </c>
-      <c r="H28" s="29"/>
-      <c r="I28" s="30">
-        <v>9</v>
-      </c>
-      <c r="J28" s="29"/>
-      <c r="K28" s="29" t="inlineStr">
+      <c r="J28" s="26"/>
+      <c r="K28" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">approve adjusted</t>
         </is>
       </c>
-      <c r="L28" s="29" t="inlineStr">
+      <c r="L28" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness (via assistant)</t>
         </is>
       </c>
-      <c r="M28" s="29" t="inlineStr">
+      <c r="M28" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-30 07:34:12</t>
         </is>
       </c>
-      <c r="N28" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Owner 30 Sep 2026: rate set by team/date rule (Sunbet set-up = event; same team same day = same rate). See row note.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B29" s="29">
-        <v>10299</v>
-      </c>
-      <c r="C29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thandanani Nkala</t>
-        </is>
-      </c>
-      <c r="D29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29</t>
-        </is>
-      </c>
-      <c r="E29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
-        </is>
-      </c>
-      <c r="G29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
-        </is>
-      </c>
-      <c r="H29" s="29"/>
-      <c r="I29" s="30">
-        <v>9</v>
-      </c>
-      <c r="J29" s="29"/>
-      <c r="K29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness (via assistant)</t>
-        </is>
-      </c>
-      <c r="M29" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-30 07:34:12</t>
-        </is>
-      </c>
-      <c r="N29" s="29" t="inlineStr">
+      <c r="N28" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">Owner 30 Sep 2026: rate set by team/date rule (Sunbet set-up = event; same team same day = same rate). See row note.</t>
         </is>
@@ -13292,7 +13236,7 @@
         <v>600</v>
       </c>
       <c r="G17" s="4">
-        <v>250</v>
+        <v>360</v>
       </c>
       <c r="H17" s="4">
         <v>240</v>
@@ -13344,7 +13288,7 @@
         <v>500</v>
       </c>
       <c r="G18" s="4">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="H18" s="4">
         <v>0</v>

</xml_diff>

<commit_message>
Auditor deduction note: amount-first lines adding to TOTAL DEDUCTED (owner format, v2026-10-01-3)
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
@@ -8957,7 +8957,7 @@
       </c>
       <c r="AB7" s="36"/>
     </row>
-    <row r="8" ht="97" customHeight="1">
+    <row r="8" ht="124" customHeight="1">
       <c r="A8" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Erick Mpho Molefe</t>
@@ -9043,9 +9043,10 @@
       </c>
       <c r="AB8" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
-2. LOAN #1 R2 000,00 given 2026-08-08 (car repair): R250,00 deducted this week; R250,00 still owing — carried to the next payroll.
-3. LOAN #7 R500,00 given 2026-09-22 (cash advance requested by WhatsApp): R250,00 deducted this week; R250,00 still owing — carried to the next payroll.</t>
+          <t xml:space="preserve">1  Car Payment (vehicle, fixed weekly): taking 1000
+2  Car repair (loan 2026-08-08): 2000, taking 250 — 250 still owing
+3  Cash advance requested by WhatsApp (loan 2026-09-22): 500, taking 250 — 250 still owing
+= TOTAL DEDUCTED 1500</t>
         </is>
       </c>
     </row>
@@ -9135,7 +9136,7 @@
       </c>
       <c r="AB9" s="36"/>
     </row>
-    <row r="10" ht="124" customHeight="1">
+    <row r="10" ht="151" customHeight="1">
       <c r="A10" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
@@ -9221,10 +9222,11 @@
       </c>
       <c r="AB10" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. FIXED R260,00/week — Eggs, every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
-2. LOAN #2 R900,00 given 2026-08-11 (cash advance): R350,00 deducted this week; now fully repaid — CLOSED, nothing further.
-3. LOAN #3 R600,00 given 2026-08-16 (cash advance): R150,00 deducted this week (only what was left); now fully repaid — CLOSED, nothing further.
-4. LOAN #6 R600,00 given 2026-09-01 (children's school trip): R240,00 deducted this week; R360,00 still owing — carried to the next payroll.</t>
+          <t xml:space="preserve">1  Eggs (fixed weekly): taking 260
+2  Cash advance (loan 2026-08-11): 900, taking 350 — paid off, closed
+3  Cash advance (loan 2026-08-16): 600, taking 150 — paid off, closed
+4  Children's school trip (loan 2026-09-01): 600, taking 240 — 360 still owing
+= TOTAL DEDUCTED 1000</t>
         </is>
       </c>
     </row>
@@ -9314,7 +9316,7 @@
       </c>
       <c r="AB11" s="36"/>
     </row>
-    <row r="12" ht="43" customHeight="1">
+    <row r="12" ht="70" customHeight="1">
       <c r="A12" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Joshua Motsamai Nteo</t>
@@ -9400,7 +9402,8 @@
       </c>
       <c r="AB12" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-09-26, ongoing until the owner ends it. Not a loan.</t>
+          <t xml:space="preserve">1  Car Payment (vehicle, fixed weekly): taking 1000
+= TOTAL DEDUCTED 1000</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10496,7 @@
       </c>
       <c r="N8" s="36"/>
     </row>
-    <row r="9" ht="97" customHeight="1">
+    <row r="9" ht="124" customHeight="1">
       <c r="A9" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Erick Mpho Molefe</t>
@@ -10537,9 +10540,10 @@
       </c>
       <c r="N9" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
-2. LOAN #1 R2 000,00 given 2026-08-08 (car repair): R250,00 deducted this week; R250,00 still owing — carried to the next payroll.
-3. LOAN #7 R500,00 given 2026-09-22 (cash advance requested by WhatsApp): R250,00 deducted this week; R250,00 still owing — carried to the next payroll.</t>
+          <t xml:space="preserve">1  Car Payment (vehicle, fixed weekly): taking 1000
+2  Car repair (loan 2026-08-08): 2000, taking 250 — 250 still owing
+3  Cash advance requested by WhatsApp (loan 2026-09-22): 500, taking 250 — 250 still owing
+= TOTAL DEDUCTED 1500</t>
         </is>
       </c>
     </row>
@@ -10587,7 +10591,7 @@
       </c>
       <c r="N10" s="36"/>
     </row>
-    <row r="11" ht="124" customHeight="1">
+    <row r="11" ht="151" customHeight="1">
       <c r="A11" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
@@ -10631,10 +10635,11 @@
       </c>
       <c r="N11" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. FIXED R260,00/week — Eggs, every week since 2026-08-01, ongoing until the owner ends it. Not a loan.
-2. LOAN #2 R900,00 given 2026-08-11 (cash advance): R350,00 deducted this week; now fully repaid — CLOSED, nothing further.
-3. LOAN #3 R600,00 given 2026-08-16 (cash advance): R150,00 deducted this week (only what was left); now fully repaid — CLOSED, nothing further.
-4. LOAN #6 R600,00 given 2026-09-01 (children's school trip): R240,00 deducted this week; R360,00 still owing — carried to the next payroll.</t>
+          <t xml:space="preserve">1  Eggs (fixed weekly): taking 260
+2  Cash advance (loan 2026-08-11): 900, taking 350 — paid off, closed
+3  Cash advance (loan 2026-08-16): 600, taking 150 — paid off, closed
+4  Children's school trip (loan 2026-09-01): 600, taking 240 — 360 still owing
+= TOTAL DEDUCTED 1000</t>
         </is>
       </c>
     </row>
@@ -10682,7 +10687,7 @@
       </c>
       <c r="N12" s="36"/>
     </row>
-    <row r="13" ht="43" customHeight="1">
+    <row r="13" ht="70" customHeight="1">
       <c r="A13" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Joshua Motsamai Nteo</t>
@@ -10726,7 +10731,8 @@
       </c>
       <c r="N13" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIXED R1 000,00/week — Car Payment (vehicle: held from wages weekly, paid over to the worker on the 25th of each month), every week since 2026-09-26, ongoing until the owner ends it. Not a loan.</t>
+          <t xml:space="preserve">1  Car Payment (vehicle, fixed weekly): taking 1000
+= TOTAL DEDUCTED 1000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auditor note = owner's table: Line | item | Owing before | Taken (v2026-10-01-4)
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-26_to_2026-10-02_AUDITOR.xlsx
@@ -8957,7 +8957,7 @@
       </c>
       <c r="AB7" s="36"/>
     </row>
-    <row r="8" ht="124" customHeight="1">
+    <row r="8" ht="97" customHeight="1">
       <c r="A8" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Erick Mpho Molefe</t>
@@ -9043,10 +9043,9 @@
       </c>
       <c r="AB8" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1  Car Payment (vehicle, fixed weekly): taking 1000
-2  Car repair (loan 2026-08-08): 2000, taking 250 — 250 still owing
-3  Cash advance requested by WhatsApp (loan 2026-09-22): 500, taking 250 — 250 still owing
-= TOTAL DEDUCTED 1500</t>
+          <t xml:space="preserve">1  Car Payment (fixed)  |  Owing before: —  |  Taken: R1000
+2  #1 car repair R2000  |  Owing before: R500  |  Taken: R250
+3  #7 cash advance requested by WhatsApp R500  |  Owing before: R500  |  Taken: R250</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9135,7 @@
       </c>
       <c r="AB9" s="36"/>
     </row>
-    <row r="10" ht="151" customHeight="1">
+    <row r="10" ht="124" customHeight="1">
       <c r="A10" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
@@ -9222,11 +9221,10 @@
       </c>
       <c r="AB10" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1  Eggs (fixed weekly): taking 260
-2  Cash advance (loan 2026-08-11): 900, taking 350 — paid off, closed
-3  Cash advance (loan 2026-08-16): 600, taking 150 — paid off, closed
-4  Children's school trip (loan 2026-09-01): 600, taking 240 — 360 still owing
-= TOTAL DEDUCTED 1000</t>
+          <t xml:space="preserve">1  Eggs (fixed)  |  Owing before: —  |  Taken: R260
+2  #2 cash advance R900  |  Owing before: R350  |  Taken: R350
+3  #3 cash advance R600  |  Owing before: R150  |  Taken: R150
+4  #6 children's school trip R600  |  Owing before: R600  |  Taken: R240</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9314,7 @@
       </c>
       <c r="AB11" s="36"/>
     </row>
-    <row r="12" ht="70" customHeight="1">
+    <row r="12" ht="43" customHeight="1">
       <c r="A12" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Joshua Motsamai Nteo</t>
@@ -9402,8 +9400,7 @@
       </c>
       <c r="AB12" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1  Car Payment (vehicle, fixed weekly): taking 1000
-= TOTAL DEDUCTED 1000</t>
+          <t xml:space="preserve">1  Car Payment (fixed)  |  Owing before: —  |  Taken: R1000</t>
         </is>
       </c>
     </row>
@@ -10496,7 +10493,7 @@
       </c>
       <c r="N8" s="36"/>
     </row>
-    <row r="9" ht="124" customHeight="1">
+    <row r="9" ht="97" customHeight="1">
       <c r="A9" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Erick Mpho Molefe</t>
@@ -10540,10 +10537,9 @@
       </c>
       <c r="N9" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1  Car Payment (vehicle, fixed weekly): taking 1000
-2  Car repair (loan 2026-08-08): 2000, taking 250 — 250 still owing
-3  Cash advance requested by WhatsApp (loan 2026-09-22): 500, taking 250 — 250 still owing
-= TOTAL DEDUCTED 1500</t>
+          <t xml:space="preserve">1  Car Payment (fixed)  |  Owing before: —  |  Taken: R1000
+2  #1 car repair R2000  |  Owing before: R500  |  Taken: R250
+3  #7 cash advance requested by WhatsApp R500  |  Owing before: R500  |  Taken: R250</t>
         </is>
       </c>
     </row>
@@ -10591,7 +10587,7 @@
       </c>
       <c r="N10" s="36"/>
     </row>
-    <row r="11" ht="151" customHeight="1">
+    <row r="11" ht="124" customHeight="1">
       <c r="A11" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
@@ -10635,11 +10631,10 @@
       </c>
       <c r="N11" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1  Eggs (fixed weekly): taking 260
-2  Cash advance (loan 2026-08-11): 900, taking 350 — paid off, closed
-3  Cash advance (loan 2026-08-16): 600, taking 150 — paid off, closed
-4  Children's school trip (loan 2026-09-01): 600, taking 240 — 360 still owing
-= TOTAL DEDUCTED 1000</t>
+          <t xml:space="preserve">1  Eggs (fixed)  |  Owing before: —  |  Taken: R260
+2  #2 cash advance R900  |  Owing before: R350  |  Taken: R350
+3  #3 cash advance R600  |  Owing before: R150  |  Taken: R150
+4  #6 children's school trip R600  |  Owing before: R600  |  Taken: R240</t>
         </is>
       </c>
     </row>
@@ -10687,7 +10682,7 @@
       </c>
       <c r="N12" s="36"/>
     </row>
-    <row r="13" ht="70" customHeight="1">
+    <row r="13" ht="43" customHeight="1">
       <c r="A13" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">Joshua Motsamai Nteo</t>
@@ -10731,8 +10726,7 @@
       </c>
       <c r="N13" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1  Car Payment (vehicle, fixed weekly): taking 1000
-= TOTAL DEDUCTED 1000</t>
+          <t xml:space="preserve">1  Car Payment (fixed)  |  Owing before: —  |  Taken: R1000</t>
         </is>
       </c>
     </row>

</xml_diff>